<commit_message>
Doc: Troca do arquivo de custos antigo para o novo
</commit_message>
<xml_diff>
--- a/Arquivos-Escopo/custosAgroflux.xlsx
+++ b/Arquivos-Escopo/custosAgroflux.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52065354-3ACA-48FE-8280-AECA372C4CFC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E77748-7F4F-411D-881F-30118CCA8AC9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" activeTab="1" xr2:uid="{DB42DB59-C03E-4685-9717-9A41DF19113F}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{DB42DB59-C03E-4685-9717-9A41DF19113F}"/>
   </bookViews>
   <sheets>
     <sheet name="Custo de projeto completo " sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="53">
   <si>
     <t>CUSTOS DE DESENVOLVIMENTO</t>
   </si>
@@ -171,15 +171,6 @@
     <t>Custo Anual</t>
   </si>
   <si>
-    <t>Desenvolvedor Back-end - Júnior</t>
-  </si>
-  <si>
-    <t>Analista de Qualidade (QA) - Júnior</t>
-  </si>
-  <si>
-    <t>Gerente de Projetos - Júnior</t>
-  </si>
-  <si>
     <t>2. Custos de Infraestrutura</t>
   </si>
   <si>
@@ -213,7 +204,10 @@
     <t>Desenvolvedor Front-end - SÊNIOR</t>
   </si>
   <si>
-    <t>Desenvolvedor Back-end  - Júnior</t>
+    <t>Valor hora</t>
+  </si>
+  <si>
+    <t>Desenvolvedor Front-end  - SÊNIOR</t>
   </si>
 </sst>
 </file>
@@ -315,7 +309,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -375,12 +369,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -397,49 +402,7 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -461,7 +424,67 @@
     <xf numFmtId="44" fontId="0" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -805,24 +828,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -852,7 +875,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="2">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="D4" s="2">
         <v>6</v>
@@ -862,33 +885,33 @@
       </c>
       <c r="F4" s="3">
         <f>C4*D4*E4</f>
-        <v>42000</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2">
         <v>1</v>
       </c>
       <c r="C5" s="2">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="D5" s="2">
         <v>6</v>
       </c>
       <c r="E5" s="3">
-        <v>28</v>
+        <v>41.66</v>
       </c>
       <c r="F5" s="3">
         <f>C5*D5*E5</f>
-        <v>33600</v>
+        <v>54991.199999999997</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B6" s="2">
         <v>2</v>
@@ -903,13 +926,13 @@
         <v>45</v>
       </c>
       <c r="F6" s="3">
-        <f t="shared" ref="F6:F8" si="0">C6*D6*E6</f>
-        <v>54000</v>
+        <f>C6*D6*E6*B6</f>
+        <v>108000</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B7" s="2">
         <v>2</v>
@@ -924,8 +947,8 @@
         <v>60</v>
       </c>
       <c r="F7" s="3">
-        <f>C7*D7*E7</f>
-        <v>72000</v>
+        <f>C7*D7*E7*B7</f>
+        <v>144000</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -945,30 +968,30 @@
         <v>25</v>
       </c>
       <c r="F8" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="F6:F8" si="0">C8*D8*E8</f>
         <v>30000</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
       <c r="F9" s="4">
         <f>SUM(F4:F8)</f>
-        <v>231600</v>
+        <v>383191.2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -995,7 +1018,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="3">
-        <f t="shared" ref="D14:D19" si="1">B14*C14</f>
+        <f>B14*C14</f>
         <v>18000</v>
       </c>
     </row>
@@ -1010,7 +1033,7 @@
         <v>6</v>
       </c>
       <c r="D15" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D14:D19" si="1">B15*C15</f>
         <v>6000</v>
       </c>
     </row>
@@ -1075,21 +1098,21 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="4">
         <f>SUM(D14:D19)</f>
         <v>44400</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="23"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
@@ -1132,7 +1155,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="8" t="s">
         <v>30</v>
       </c>
       <c r="B28" s="4">
@@ -1141,45 +1164,45 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="17"/>
+      <c r="B30" s="16"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="25" t="s">
+      <c r="A31" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="26">
+      <c r="B31" s="12">
         <f>F9</f>
-        <v>231600</v>
+        <v>383191.2</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="28">
+      <c r="B32" s="14">
         <f>D20</f>
         <v>44400</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="27" t="s">
+      <c r="A33" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="28">
+      <c r="B33" s="14">
         <f>B28</f>
         <v>8500</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="27" t="s">
+      <c r="A34" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="29">
+      <c r="B34" s="15">
         <f>SUM(B31:B33)</f>
-        <v>284500</v>
+        <v>436091.2</v>
       </c>
     </row>
   </sheetData>
@@ -1199,124 +1222,147 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDB5F906-94D0-4D38-BB69-71482984B91D}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.88671875" customWidth="1"/>
     <col min="2" max="2" width="16.6640625" customWidth="1"/>
     <col min="3" max="3" width="13.5546875" customWidth="1"/>
     <col min="4" max="4" width="15.5546875" customWidth="1"/>
+    <col min="5" max="5" width="20.44140625" customWidth="1"/>
+    <col min="6" max="6" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="35"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>37</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B4" s="2">
         <v>38</v>
       </c>
       <c r="C4" s="3">
-        <v>2200</v>
+        <v>45</v>
       </c>
       <c r="D4" s="3">
-        <f>C4*12</f>
-        <v>26400</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1710</v>
+      </c>
+      <c r="E4" s="3">
+        <f>B4*C4*12</f>
+        <v>20520</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B5" s="2">
         <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>2800</v>
+        <v>60</v>
       </c>
       <c r="D5" s="3">
-        <f>C5*12</f>
-        <v>33600</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1200</v>
+      </c>
+      <c r="E5" s="3">
+        <f>B5*C5*12</f>
+        <v>14400</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="B6" s="2">
         <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>2000</v>
+        <v>41.66</v>
       </c>
       <c r="D6" s="3">
-        <f>C6*12</f>
-        <v>24000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+        <v>829.03</v>
+      </c>
+      <c r="E6" s="3">
+        <f>B6*C6*12</f>
+        <v>9998.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2">
         <v>10</v>
       </c>
       <c r="C7" s="3">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="D7" s="3">
-        <f>C7*12</f>
-        <v>1080</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="E7" s="3">
+        <f>B7*C7*12</f>
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="7">
-        <f>SUM(D4:D7)</f>
-        <v>85080</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="7">
+        <f>SUM(E4:E7)</f>
+        <v>49118.400000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>11</v>
       </c>
@@ -1327,7 +1373,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>18</v>
       </c>
@@ -1339,7 +1385,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>17</v>
       </c>
@@ -1351,7 +1397,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>16</v>
       </c>
@@ -1363,7 +1409,7 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>19</v>
       </c>
@@ -1376,21 +1422,21 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="12"/>
+      <c r="A17" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="27"/>
       <c r="C17" s="7">
         <f>SUM(C13:C16)</f>
         <v>16440</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
+      <c r="A19" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
@@ -1429,7 +1475,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B23" s="3">
         <v>500</v>
@@ -1440,62 +1486,62 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B24" s="12"/>
+      <c r="A24" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="27"/>
       <c r="C24" s="7">
         <f>SUM(C21:C23)</f>
         <v>14340</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="B27" s="22"/>
+      <c r="A27" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" s="26"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="B28" s="24">
-        <f>D8</f>
-        <v>85080</v>
+      <c r="A28" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B28" s="10">
+        <f>E8</f>
+        <v>49118.400000000001</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="24">
+      <c r="A29" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B29" s="10">
         <f>C17</f>
         <v>16440</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="B30" s="24">
+      <c r="A30" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" s="10">
         <f>C24</f>
         <v>14340</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="23" t="s">
+      <c r="A31" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="24">
+      <c r="B31" s="10">
         <f>SUM(B28:B30)</f>
-        <v>115860</v>
+        <v>79898.399999999994</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A8:D8"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A8:C8"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A19:C19"/>

</xml_diff>